<commit_message>
Add map_to_questionnaire.py: transfer data into REDI Mapping Questionnaire Excel format
Co-authored-by: MartinaIjaz <MartinaIjaz@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/primer_so_duplikati.xlsx
+++ b/primer_so_duplikati.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:Z8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,6 +452,101 @@
           <t>Општина</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Земја</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Пол</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Година на раѓање</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Образование</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Рома</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Врска со ромска заедница</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Бизнис</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Адреса на бизнис</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Опис на бизнис</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Сектор</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Регистриран</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Датум на регистрација</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Вработени</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>Фаза I</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Година на поддршка</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>Тип на услуга</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>Бизнис клуб</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>Кредит</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>Информиран</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -474,7 +569,11 @@
           <t>070 111 222</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>marko@mk.com</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>ул. Мир 5</t>
@@ -483,6 +582,91 @@
       <c r="G2" t="inlineStr">
         <is>
           <t>Центар</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Македонија</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>М</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>1985</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Факултет</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Петров Трговија</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>ул. Мир 5</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Трговија со мешана стока</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Трговија</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>2015-06-01</t>
+        </is>
+      </c>
+      <c r="T2" t="n">
+        <v>3</v>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="V2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Маркетинг и промоција</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>Да</t>
         </is>
       </c>
     </row>
@@ -502,14 +686,109 @@
           <t>2021-06-15</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>070 777 888</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>ana@mk.com</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>ул. Цвет 7</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Центар</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Македонија</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Ж</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>1990</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Магистер</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Ана Салон</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>ул. Цвет 7</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Фризерски и козметички салон</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Убавина и здравје</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>2018-03-15</t>
+        </is>
+      </c>
+      <c r="T3" t="n">
+        <v>1</v>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Не</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>Дигитализација на бизнис</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>Не</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -532,7 +811,11 @@
           <t>071 333 444</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>petar@mk.com</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
           <t>ул. Роза 12</t>
@@ -541,287 +824,569 @@
       <c r="G4" t="inlineStr">
         <is>
           <t>Карпош</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Македонија</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>М</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>1978</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Средно</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Не</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Сопруг е Ром</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Стојанов Градба</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>ул. Роза 12</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Градежни работи и реновирање</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Градежништво</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>2010-11-20</t>
+        </is>
+      </c>
+      <c r="T4" t="n">
+        <v>5</v>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="V4" t="n">
+        <v>2021</v>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>Пристап до грант</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>Можеби</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>Не</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Марко</t>
+          <t>Елена</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Петров</t>
+          <t>Велкова</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2022-03-10</t>
+          <t>2024-02-28</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>marko@mk.com</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
+          <t>elena@mk.com</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>ул. Езеро 1</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Центар</t>
+          <t>Гази Баба</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Македонија</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Ж</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>1995</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Факултет</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Велкова Угостителство</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>ул. Езеро 1</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Кафе-бар и угостителство</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Туризам и угостителство</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Не</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Не</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>Регистрација на бизнис</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>Не</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>Да</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Сара</t>
+          <t>Никола</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Ристова</t>
+          <t>Јовиќ</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2020-11-05</t>
+          <t>2022-08-01</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>072 555 666</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr"/>
+          <t>075 999 000</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>nikola@mk.com</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>ул. Сонце 3</t>
+          <t>ул. Планин 9</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Аеродром</t>
+          <t>Бит Пазар</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Македонија</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>М</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>1982</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Средно</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Јовиќ Транспорт</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>ул. Планин 9</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Превоз на патници и стоки</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Транспорт</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>2016-07-05</t>
+        </is>
+      </c>
+      <c r="T6" t="n">
+        <v>2</v>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Не</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>Бизнис консалтинг</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>Не</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>Не</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>Не</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Ана</t>
+          <t>Сара</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Иванова</t>
+          <t>Ристова</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2021-06-15</t>
+          <t>2020-11-05</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>070 777 888</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
+          <t>072 555 666</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>sara@mk.com</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>ул. Цвет 7</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
+          <t>ул. Сонце 3</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Аеродром</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Македонија</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Ж</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>1988</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Факултет</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Не</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Партнер е Ром</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Ристова Козметика</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>ул. Сонце 3</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Козметички третмани и нега</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Убавина и здравје</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Не</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="n">
+        <v>1</v>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Не</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>Регистрација на бизнис</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>Не</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Елена</t>
+          <t>Томе</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Велкова</t>
+          <t>Спасов</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2024-02-28</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
+          <t>2019-09-12</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>078 333 444</t>
+        </is>
+      </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>elena@mk.com</t>
+          <t>tome@mk.com</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>ул. Езеро 1</t>
+          <t>ул. Гора 2</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Гази Баба</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Никола</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Јовиќ</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>2022-08-01</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>075 999 000</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>ул. Планин 9</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Бит Пазар</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Петар</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Стојанов</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>2023-01-20</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>petar@mk.com</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Сара</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Ристова</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>2020-11-05</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>sara@mk.com</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Аеродром</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Никола</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Јовиќ</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>2022-08-01</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>075 111 222</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>nikola@mk.com</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Бит Пазар</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Томе</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Спасов</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>2019-09-12</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>078 333 444</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>tome@mk.com</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
+          <t>Ѓорче Петров</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Македонија</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>М</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>1975</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Занаетчиско</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Спасов Занает</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
         <is>
           <t>ул. Гора 2</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Ѓорче</t>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Изработка на метални конструкции</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Производство</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>2005-02-28</t>
+        </is>
+      </c>
+      <c r="T8" t="n">
+        <v>4</v>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="V8" t="n">
+        <v>2020</v>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>Менторство еден-на-еден</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>Можеби</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>Да</t>
         </is>
       </c>
     </row>

</xml_diff>